<commit_message>
Record the Wikidata vernacular-name fill as applied
wikidata-species moves from assessed to partial: the species-import
question is still correctly undecided (downstream of the
bacteria-and-viruses hold), but the VernacularName.tsv sidecar is now
applied -- 39,322 commonName filled, see the previous commit. Media
and Distribution remain unapplied for their own separate reasons
(licence lookup, place-name resolution). Synced sourcesManifest.py,
bacteria-and-viruses.md and the linked data-sources.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reports/data-sources.xlsx
+++ b/docs/reports/data-sources.xlsx
@@ -42,7 +42,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +57,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -96,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -116,6 +121,9 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -483,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -559,110 +567,120 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>assessed</t>
+          <t>partial</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>assessed</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>refused</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B10" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Triage verdict (candidate datasets, resolved)</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>take / applied</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>14</v>
+          <t>Triage verdict (candidate datasets, resolved)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>declined / superseded</t>
+          <t>take / applied</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>declined / superseded</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>other</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B16" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Total manifest entries</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>69</v>
-      </c>
-    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Total candidate-triage rows</t>
+          <t>Total manifest entries</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>32</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Total candidate-triage rows</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Rows where the table verdict conflicted with its own prose</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B20" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
         <is>
           <t>(see 'Candidate triage log', Verdict (resolved) + Notes columns)</t>
         </is>
@@ -1994,306 +2012,306 @@
     <row r="37" ht="60" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-1021</t>
+          <t>wikidata-species</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Orthoptera Species File, ChecklistBank edition (dataset 1021)</t>
+          <t>Wikidata Species (ChecklistBank dataset 314569)</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d388; version Oct 2026, issued 2026-10-01</t>
+          <t>DOI 10.48580/dgx38; version 2026-08-02; contact Markus Doering (GBIF); generated by CatalogueOfLife/coldp-generator</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/1021</t>
+          <t>https://www.checklistbank.org/dataset/314569</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>CC BY</t>
+          <t>CC0</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>assessed</t>
+          <t>partial</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>NOT taken. 30,890 name usages, 88.3% of a 600-name sample already held -- the lowest overlap in its batch, which reads as an opening but is not one: this is the current release of manifest `orthoptera`, which we applied from GBIF at 28,081 species, and the 27,194 species carrying sourcedFrom 'orthoptera species file' come from it. What is left is one release cycle of taxonomic churn in one group, not names we are missing. Re-importing as a replacement and diffing is the only clean way to take it.</t>
+          <t>SPECIES IMPORT NOT TAKEN, and not yet a decision either -- see below, the question is downstream of the bacteria-and-viruses hold. The commonName sidecar IS applied; see VernacularName.tsv further down. Measured with scripts/overlapReport.py, which uses the importers' own held/new test rather than a raw string comparison: 3,207,163 accepted species, of which 1,395,018 (43.5%) we already hold and 1,811,989 (56.5%) are new. Of the new ones 91% resolve both a family and an order and would land in a real family rather than an Incertae sedis placeholder. Zero duplicates within the archive, 156 non-binomials. Taken, this would roughly double animalia and bring prokaryotes and viruses with it. CC0, so licensing is not an obstacle. It does NOT resolve the bacteria-and-viruses rank question: Wikidata carries the same 17 kingdom-rank clades COL does (Bacillati, Pseudomonadati, Orthornavirae, Heunggongvirae, ...) because it is built from the same upstream, and 1,612,751 of the new species have no parent at all. See docs/bacteria-and-viruses.md for the options. First archive in the ColDP format we hold, and first to exercise scripts/coldp.py. RE-CHECKED 2026-10-10: species-import question still correctly undecided -- it is downstream of the bacteria-and-viruses hold, which is unchanged (GTDB has since settled the bacterial rank; viruses are still blocked on ICTV). The 2026-10-04 measurement was already taken after Animalia Stage 2, so the ~135k species added since (ITIS, BOLD, GLI, Craneflies, Reptiles) shave a little off 1,811,989 but do not change the shape of the decision -- not worth re-measuring on its own. SIDECAR FINDING, measured 2026-10-10 against the held tree (scripts/tree.py, one walk, 2,531,312 held names): the same archive's sidecar tables carry real content the species-count note above never looked at, and most of each one lands on species we already hold -- this is an enrichment question, not an import one, so none of it waits on the bacteria-and-viruses hold. Media.tsv: 340,025 distinct taxa, 192,847 held, of which 110,224 already have an image in wiki-images.json and 82,623 do not -- but 663,287 of 664,930 rows (99.75%) carry no licence string at all, so that gap needs a per-image Commons licence lookup before anything is written, not a straight copy. VernacularName.tsv: APPLIED 2026-10-10 by scripts/enrichCommonNamesFromWikidata.py -- 816,277 rows in 108 languages, filtered to species-rank taxa and en/blank the way scripts/enrichCommonNamesFromGbif.py filters GBIF's table, plus one filter neither needed: 31 candidates that were just the binomial re-capitalised, not a translation, found by sampling before applying. **39,322 commonName filled** across 2,150 files (animalia 21,960, plantae 15,457, fungi 1,903, chromista 2) -- bigger than the 23,287 the GBIF Backbone pass filled. Idempotent, verified. Distribution.tsv: 293,850 rows, 103,213 distinct taxa, 66,815 held, 35,043 already have continents, 31,772 do not; 83.9% of rows are free-text place names needing resolution (the USDA PLANTS problem again) and 16.1% are ISO codes mappable through the existing CC2CONT table today -- roughly 5,100 of the 31,772 need no new plumbing. Not yet done: writing the importer. Vernacular is the obvious first pick -- biggest clean gap, smallest new code.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="60" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-1022</t>
+          <t>checklistbank-1021</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Parhost World Database of Fleas (dataset 1022)</t>
+          <t>Orthoptera Species File, ChecklistBank edition (dataset 1021)</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d389; version 2, issued 2005-11-14</t>
+          <t>DOI 10.48580/d388; version Oct 2026, issued 2026-10-01</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/1022</t>
+          <t>https://www.checklistbank.org/dataset/1021</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="F38" s="7" t="inlineStr">
+          <t>CC BY</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>NOT taken. 2,047 name usages, 96.7% of a 600-name sample already held. ChecklistBank records the licence as 'other', so permission is not established -- which settles it independently of the weak coverage argument.</t>
+          <t>NOT taken. 30,890 name usages, 88.3% of a 600-name sample already held -- the lowest overlap in its batch, which reads as an opening but is not one: this is the current release of manifest `orthoptera`, which we applied from GBIF at 28,081 species, and the 27,194 species carrying sourcedFrom 'orthoptera species file' come from it. What is left is one release cycle of taxonomic churn in one group, not names we are missing. Re-importing as a replacement and diffing is the only clean way to take it.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="60" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-1023</t>
+          <t>checklistbank-1022</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Phyllachorales (dataset 1023)</t>
+          <t>Parhost World Database of Fleas (dataset 1022)</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d38b; issued 2017-10-27</t>
+          <t>DOI 10.48580/d389; version 2, issued 2005-11-14</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/1023</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr"/>
-      <c r="F39" s="7" t="inlineStr">
+          <t>https://www.checklistbank.org/dataset/1022</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>NOT taken. 1,311 name usages, 95.8% of a 600-name sample already held. ChecklistBank records NO licence for this dataset, which is not the same as a permissive one and is not usable on evidence.</t>
+          <t>NOT taken. 2,047 name usages, 96.7% of a 600-name sample already held. ChecklistBank records the licence as 'other', so permission is not established -- which settles it independently of the weak coverage argument.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="60" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-1024</t>
+          <t>checklistbank-1023</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>World Checklist of Selected Plant Families (WCSP)</t>
+          <t>Phyllachorales (dataset 1023)</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d38c</t>
+          <t>DOI 10.48580/d38b; issued 2017-10-27</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/1024</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>CC BY 4.0</t>
-        </is>
-      </c>
-      <c r="F40" s="7" t="inlineStr">
+          <t>https://www.checklistbank.org/dataset/1023</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr"/>
+      <c r="F40" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>NOT TAKEN, vintage. 416,075 name usages, all 116 families held, accepted-species count 120,288 -- and the edition is 2017-08-25, nine years old, against WFO Plant List 2026-06 (CC0, applied), POWO and the World Checklist of Vascular Plants (applied). The same verdict as Tropicos: importing older nomenclatural data over newer is a taxonomy decision, not a data one. Its archive endpoint also returns HTTP 404, so it cannot be measured offline at all</t>
+          <t>NOT taken. 1,311 name usages, 95.8% of a 600-name sample already held. ChecklistBank records NO licence for this dataset, which is not the same as a permissive one and is not usable on evidence.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="60" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-1025</t>
+          <t>checklistbank-1024</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Rhytismatales (dataset 1025)</t>
+          <t>World Checklist of Selected Plant Families (WCSP)</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d38d; issued 2017-10-27</t>
+          <t>DOI 10.48580/d38c</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/1025</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr"/>
-      <c r="F41" s="7" t="inlineStr">
+          <t>https://www.checklistbank.org/dataset/1024</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>CC BY 4.0</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>NOT taken. 769 name usages, 96.7% of a 600-name sample already held. No licence stated, as 1023.</t>
+          <t>NOT TAKEN, vintage. 416,075 name usages, all 116 families held, accepted-species count 120,288 -- and the edition is 2017-08-25, nine years old, against WFO Plant List 2026-06 (CC0, applied), POWO and the World Checklist of Vascular Plants (applied). The same verdict as Tropicos: importing older nomenclatural data over newer is a taxonomy decision, not a data one. Its archive endpoint also returns HTTP 404, so it cannot be measured offline at all</t>
         </is>
       </c>
     </row>
     <row r="42" ht="60" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-1026</t>
+          <t>checklistbank-1025</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>ScaleNet, Systematic Database of the Scale Insects of the World (dataset 1026)</t>
+          <t>Rhytismatales (dataset 1025)</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d38f; version Dec 2004, issued 2004-12-05</t>
+          <t>DOI 10.48580/d38d; issued 2017-10-27</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/1026</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>CC BY</t>
-        </is>
-      </c>
-      <c r="F42" s="7" t="inlineStr">
+          <t>https://www.checklistbank.org/dataset/1025</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr"/>
+      <c r="F42" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>NOT taken. 7,074 name usages, 83.7% of a 600-name sample held -- the largest miss in its batch at 16.3%, and still declined. Same grounds as LepIndex (1018): a twenty-year-old circumscription, so much of what it would add is obsolete names rather than missing taxa, and importing those is a taxonomy decision rather than a data one. Worth revisiting only alongside LepIndex if we decide to take synonym coverage instead of accepted taxa alone.</t>
+          <t>NOT taken. 769 name usages, 96.7% of a 600-name sample already held. No licence stated, as 1023.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="60" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-1028</t>
+          <t>checklistbank-1026</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Species Fungorum, Index Fungorum API crawl (dataset 1028)</t>
+          <t>ScaleNet, Systematic Database of the Scale Insects of the World (dataset 1026)</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d38h; version 2026-09-24</t>
+          <t>DOI 10.48580/d38f; version Dec 2004, issued 2004-12-05</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>https://api.checklistbank.org/dataset/1028/archive.zip</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="inlineStr"/>
-      <c r="F43" s="7" t="inlineStr">
+          <t>https://www.checklistbank.org/dataset/1026</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>CC BY</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>NOT taken, blocked on permission rather than coverage. 541,761 name usages, three months old, and 30.1% of its species are new to us (69.9% held over 70,961 measured) with 85.3% of its families held -- on the numbers the second-best source in its batch. ChecklistBank records NO licence for it, the same position as 1023 and 1025, and no stated terms is not permissive terms. Worth one email to Index Fungorum; the archive is otherwise ready to take. The action is on BACKLOG.md: one email to Missouri Botanical Garden, which runs Index Fungorum and Tropicos alike.</t>
+          <t>NOT taken. 7,074 name usages, 83.7% of a 600-name sample held -- the largest miss in its batch at 16.3%, and still declined. Same grounds as LepIndex (1018): a twenty-year-old circumscription, so much of what it would add is obsolete names rather than missing taxa, and importing those is a taxonomy decision rather than a data one. Worth revisiting only alongside LepIndex if we decide to take synonym coverage instead of accepted taxa alone.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="60" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-1030</t>
+          <t>checklistbank-1028</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>TicksBase (dataset 1030)</t>
+          <t>Species Fungorum, Index Fungorum API crawl (dataset 1028)</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d38k; issued 2005-06-15</t>
+          <t>DOI 10.48580/d38h; version 2026-09-24</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/1030</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>CC BY</t>
-        </is>
-      </c>
-      <c r="F44" s="7" t="inlineStr">
+          <t>https://api.checklistbank.org/dataset/1028/archive.zip</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>NOT taken. 796 name usages in total, 600 of 600 sampled species already held. The whole dataset is smaller than the sample several of its neighbours got, so 100% here is exhaustive rather than indicative. Nothing there for us.</t>
+          <t>NOT taken, blocked on permission rather than coverage. 541,761 name usages, three months old, and 30.1% of its species are new to us (69.9% held over 70,961 measured) with 85.3% of its families held -- on the numbers the second-best source in its batch. ChecklistBank records NO licence for it, the same position as 1023 and 1025, and no stated terms is not permissive terms. Worth one email to Index Fungorum; the archive is otherwise ready to take. The action is on BACKLOG.md: one email to Missouri Botanical Garden, which runs Index Fungorum and Tropicos alike.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="60" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-1032</t>
+          <t>checklistbank-1030</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Cerambycidae database</t>
+          <t>TicksBase (dataset 1030)</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d38t; version 2026-04-07</t>
+          <t>DOI 10.48580/d38k; issued 2005-06-15</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/1032</t>
+          <t>https://www.checklistbank.org/dataset/1030</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -2301,36 +2319,36 @@
           <t>CC BY</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
+      <c r="F45" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>NOT taken. Found 2026-10-10 sweeping the rest of the top-30 animalia-gaps.md families through the same search, for our #8 gap family (Cerambycidae, 23,228 missing). Measured the same way (unsharded page_all + strip_authorship + GNparser bare_name): 36,776 accepted species, 36,755 of 36,768 normalised forms (100.0%) already held, **13 new**. Declined -- same shape as Carabcat: a specialist database that COL Stage 2 already mostly absorbed.</t>
+          <t>NOT taken. 796 name usages in total, 600 of 600 sampled species already held. The whole dataset is smaller than the sample several of its neighbours got, so 100% here is exhaustive rather than indicative. Nothing there for us.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="60" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-1046</t>
+          <t>checklistbank-1032</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Global Butterfly Information System (GloBIS)</t>
+          <t>Cerambycidae database</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d38u; version Sep 2013</t>
+          <t>DOI 10.48580/d38t; version 2026-04-07</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/1046</t>
+          <t>https://www.checklistbank.org/dataset/1032</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -2338,36 +2356,36 @@
           <t>CC BY</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
+      <c r="F46" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>NOT YET DECIDED -- the one real find in the 2026-10-10 sweep. Found searching for our #30 gap family (Lycaenidae, 7,107 missing); the dataset actually covers three families (Lycaenidae, Papilionidae, Pieridae), all three already 100% held. 7,982 accepted species, 7,255 (90.9%) already held, **727 new** -- an order of magnitude more than every other 2026-10-10 lead combined (Carabcat 41 + Geometridae facility 129 + Cerambycidae 13 + Tortricidae 7 + Miridae 24 = 214). The catch is vintage: issued 2013-09, thirteen years old, the same shape as LepIndex (1018, 2012-01, hedged 'take -- biggest absolute gain' in docs/dataset-inbox.md on 2026-10-04 and never actually resolved either way). Whether a 13-year-old butterfly circumscription's novelty is real species or obsolete names superseded since is not answered by this measurement -- it is a taxonomy question, the same one Tropicos and ScaleNet were declined over, not a data one. Full species list in docs/reports/checklistbank-gap-sweep-batch2.json.</t>
+          <t>NOT taken. Found 2026-10-10 sweeping the rest of the top-30 animalia-gaps.md families through the same search, for our #8 gap family (Cerambycidae, 23,228 missing). Measured the same way (unsharded page_all + strip_authorship + GNparser bare_name): 36,776 accepted species, 36,755 of 36,768 normalised forms (100.0%) already held, **13 new**. Declined -- same shape as Carabcat: a specialist database that COL Stage 2 already mostly absorbed.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="60" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-1146</t>
+          <t>checklistbank-1046</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Carabcat database</t>
+          <t>Global Butterfly Information System (GloBIS)</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d3dk; version v.03 (08/2021)</t>
+          <t>DOI 10.48580/d38u; version Sep 2013</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/1146</t>
+          <t>https://www.checklistbank.org/dataset/1046</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
@@ -2375,36 +2393,36 @@
           <t>CC BY</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
+      <c r="F47" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>NOT taken. Found 2026-10-10 searching ChecklistBank by gap family (Carabidae, our #3 animalia gap at 31,316 missing per docs/reports/animalia-gaps.md) rather than waiting for a paste. No downloadable export exists (export.zip?format=ColDP 404s, and the POST that would generate one needs credentials this project does not have), so measured via scripts/apiOverlapReport.py's page_all, called unsharded since the 40,934 total is well under the API's 100k offset cap. The first pass (no subgenus stripping) read 58.5% as new -- the same GLI/BOLD mistake, since the misses were almost all `Genus (Subgenus) species` forms COL already holds without the parenthetical. Re-measured with strip_authorship + GNparser bare_name, the same way archiveOverlap.py does it: 40,886 of 40,934 (99.9%) already held, **41 new**. Declined -- not on licence (CC BY) or vintage (2021-08, fine for a stable group), but because the real opening is three orders of magnitude smaller than the search result's size column (108,488) suggested. COL Stage 2's animalia import already swept in most of what this independently-compiled database holds, from overlapping sources.</t>
+          <t>NOT YET DECIDED -- the one real find in the 2026-10-10 sweep. Found searching for our #30 gap family (Lycaenidae, 7,107 missing); the dataset actually covers three families (Lycaenidae, Papilionidae, Pieridae), all three already 100% held. 7,982 accepted species, 7,255 (90.9%) already held, **727 new** -- an order of magnitude more than every other 2026-10-10 lead combined (Carabcat 41 + Geometridae facility 129 + Cerambycidae 13 + Tortricidae 7 + Miridae 24 = 214). The catch is vintage: issued 2013-09, thirteen years old, the same shape as LepIndex (1018, 2012-01, hedged 'take -- biggest absolute gain' in docs/dataset-inbox.md on 2026-10-04 and never actually resolved either way). Whether a 13-year-old butterfly circumscription's novelty is real species or obsolete names superseded since is not answered by this measurement -- it is a taxonomy question, the same one Tropicos and ScaleNet were declined over, not a data one. Full species list in docs/reports/checklistbank-gap-sweep-batch2.json.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="60" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-1171</t>
+          <t>checklistbank-1146</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>On-line Systematic Catalog of Plant Bugs (Heteroptera: Miridae)</t>
+          <t>Carabcat database</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d38w; version Mar 2013</t>
+          <t>DOI 10.48580/d3dk; version v.03 (08/2021)</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/1171</t>
+          <t>https://www.checklistbank.org/dataset/1146</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
@@ -2412,36 +2430,36 @@
           <t>CC BY</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr">
+      <c r="F48" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>NOT taken. Found the same sweep, for our #14 gap family (Miridae, 11,477 missing). 11,132 accepted species, 11,108 (99.8%) held, **24 new**. Declined; negligible gain.</t>
+          <t>NOT taken. Found 2026-10-10 searching ChecklistBank by gap family (Carabidae, our #3 animalia gap at 31,316 missing per docs/reports/animalia-gaps.md) rather than waiting for a paste. No downloadable export exists (export.zip?format=ColDP 404s, and the POST that would generate one needs credentials this project does not have), so measured via scripts/apiOverlapReport.py's page_all, called unsharded since the 40,934 total is well under the API's 100k offset cap. The first pass (no subgenus stripping) read 58.5% as new -- the same GLI/BOLD mistake, since the misses were almost all `Genus (Subgenus) species` forms COL already holds without the parenthetical. Re-measured with strip_authorship + GNparser bare_name, the same way archiveOverlap.py does it: 40,886 of 40,934 (99.9%) already held, **41 new**. Declined -- not on licence (CC BY) or vintage (2021-08, fine for a stable group), but because the real opening is three orders of magnitude smaller than the search result's size column (108,488) suggested. COL Stage 2's animalia import already swept in most of what this independently-compiled database holds, from overlapping sources.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="60" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-185410</t>
+          <t>checklistbank-1171</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Online Taxonomic Facility of Geometridae</t>
+          <t>On-line Systematic Catalog of Plant Bugs (Heteroptera: Miridae)</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d9mhh; version 1.1.24.158 (2024-06-06)</t>
+          <t>DOI 10.48580/d38w; version Mar 2013</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/185410</t>
+          <t>https://www.checklistbank.org/dataset/1171</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
@@ -2449,36 +2467,36 @@
           <t>CC BY</t>
         </is>
       </c>
-      <c r="F49" s="7" t="inlineStr">
+      <c r="F49" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>NOT taken. Found 2026-10-10 the same way as checklistbank-1146, for our #5 animalia gap family (Geometridae, 24,459 missing per docs/reports/animalia-gaps.md). Same measurement method (no downloadable export; apiOverlapReport.py's page_all, unsharded, 23,793 total well under the offset cap). Geometridae has few subgenus trinomials, so the subgenus-stripping step barely moves the number (130 raw -&gt; 129 normalised misses) the way it did for Carabcat -- but the conclusion is the same: 23,613 of 23,742 (99.5%) already held, **129 new**. Declined for the same reason: the real opening is two orders of magnitude smaller than the search result's size column (52,742) suggested.</t>
+          <t>NOT taken. Found the same sweep, for our #14 gap family (Miridae, 11,477 missing). 11,132 accepted species, 11,108 (99.8%) held, **24 new**. Declined; negligible gain.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="60" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-2007</t>
+          <t>checklistbank-185410</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>IRMNG, Interim Register of Marine and Nonmarine Genera (dataset 2007)</t>
+          <t>Online Taxonomic Facility of Geometridae</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d4f8; version 2026-09-16</t>
+          <t>DOI 10.48580/d9mhh; version 1.1.24.158 (2024-06-06)</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>https://api.checklistbank.org/dataset/2007/archive.zip</t>
+          <t>https://www.checklistbank.org/dataset/185410</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
@@ -2486,110 +2504,110 @@
           <t>CC BY</t>
         </is>
       </c>
-      <c r="F50" s="7" t="inlineStr">
+      <c r="F50" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>NOT taken, and not comparable to the species sources. 269,528 accepted genera and 2 species: it is a register of genus names, so '59.9% of its genera are held' answers a different question from the rest of the batch. Its value is nomenclatural availability, which this tree does not model. Sampled at species rank before the tooling was fixed, it reported a confident 100% already-held from a two-name sample.</t>
+          <t>NOT taken. Found 2026-10-10 the same way as checklistbank-1146, for our #5 animalia gap family (Geometridae, 24,459 missing per docs/reports/animalia-gaps.md). Same measurement method (no downloadable export; apiOverlapReport.py's page_all, unsharded, 23,793 total well under the offset cap). Geometridae has few subgenus trinomials, so the subgenus-stripping step barely moves the number (130 raw -&gt; 129 normalised misses) the way it did for Carabcat -- but the conclusion is the same: 23,613 of 23,742 (99.5%) already held, **129 new**. Declined for the same reason: the real opening is two orders of magnitude smaller than the search result's size column (52,742) suggested.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="60" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-2037</t>
+          <t>checklistbank-2007</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>ZooBank (ChecklistBank bulk export)</t>
+          <t>IRMNG, Interim Register of Marine and Nonmarine Genera (dataset 2007)</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d4g9</t>
+          <t>DOI 10.48580/d4f8; version 2026-09-16</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/2037</t>
+          <t>https://api.checklistbank.org/dataset/2007/archive.zip</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>CC0 (confirmed in the archive's own eml.xml)</t>
-        </is>
-      </c>
-      <c r="F51" s="7" t="inlineStr">
+          <t>CC BY</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>NOT TAKEN, and downloaded: 81MB DwCA at archives/checklistbank-2037/archive.zip, 527,127 rows, version 2026-08-29. Measured 2026-10-09 from the archive: 275,961 names offered, 114,908 held, 160,728 NOT held, 148 of 427 families absent. The licence, the vintage and the effort are all fine; what is missing is one column. This is a NOMENCLATURAL register (ChecklistBank types it `nomenclatural`) and the DwCA writes `accepted` on every row with every acceptedNameUsageID self-referencing -- 283,875 species rows, all accepted. The ColDP edition carrying the per-name accepted/synonym split returns HTTP 406. Without it there is no way to separate the new taxa from the synonymy, so importing it is the same decision as importing COL's 2.6M synonyms, which this project holds back by policy. Only 909 of the 160,728 are ZooBank's own `Aa...` placeholder index names; the rest look like ordinary binomials (Ababactus depressus), which is what makes the register hard to refuse on data quality alone. RE-ASSESSED 2026-10-10: the archive is still on disk and still the same version. `/dataset/2037/coldp.zip` still 406s, but `/dataset/2037/export?format=ColDP` works -- it is a classification-tree JSON, not a ColDP archive -- and it carries no synonym status either: 524,236 `accepted`, 2,933 `provisionally accepted`, zero `synonym`. The flat DwCA's own taxonomicStatus agrees -- 527,106 `accepted`, 21 `invalid`, and those 21 are the only rows where id != acceptedNameUsageID, pointing not to a synonym but to an obsolete 18th-century Linnaean group name (e.g. Clupeidae -&gt; "Abdominales Linnæus, 1758") -- noise, not synonymy. So the missing column is not an export-format gap to wait out: ZooBank's data model has no accepted/synonym concept to export, in any format ChecklistBank offers. Verdict unchanged, and nothing left to re-open on</t>
+          <t>NOT taken, and not comparable to the species sources. 269,528 accepted genera and 2 species: it is a register of genus names, so '59.9% of its genera are held' answers a different question from the rest of the batch. Its value is nomenclatural availability, which this tree does not model. Sampled at species rank before the tooling was fixed, it reported a confident 100% already-held from a two-name sample.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="60" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-219318</t>
+          <t>checklistbank-2037</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>World Catalogue of the Tortricidae</t>
+          <t>ZooBank (ChecklistBank bulk export)</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/d38s; version 4.0</t>
+          <t>DOI 10.48580/d4g9</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/219318</t>
+          <t>https://www.checklistbank.org/dataset/2037</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>CC BY</t>
-        </is>
-      </c>
-      <c r="F52" s="7" t="inlineStr">
+          <t>CC0 (confirmed in the archive's own eml.xml)</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>NOT taken. Found the same sweep, for our #13 gap family (Tortricidae, 12,239 missing). 10,718 accepted species, 10,678 of 10,685 normalised forms (99.9%) held, **7 new**. Declined; 2018 vintage adds nothing -- the gain is negligible regardless.</t>
+          <t>NOT TAKEN, and downloaded: 81MB DwCA at archives/checklistbank-2037/archive.zip, 527,127 rows, version 2026-08-29. Measured 2026-10-09 from the archive: 275,961 names offered, 114,908 held, 160,728 NOT held, 148 of 427 families absent. The licence, the vintage and the effort are all fine; what is missing is one column. This is a NOMENCLATURAL register (ChecklistBank types it `nomenclatural`) and the DwCA writes `accepted` on every row with every acceptedNameUsageID self-referencing -- 283,875 species rows, all accepted. The ColDP edition carrying the per-name accepted/synonym split returns HTTP 406. Without it there is no way to separate the new taxa from the synonymy, so importing it is the same decision as importing COL's 2.6M synonyms, which this project holds back by policy. Only 909 of the 160,728 are ZooBank's own `Aa...` placeholder index names; the rest look like ordinary binomials (Ababactus depressus), which is what makes the register hard to refuse on data quality alone. RE-ASSESSED 2026-10-10: the archive is still on disk and still the same version. `/dataset/2037/coldp.zip` still 406s, but `/dataset/2037/export?format=ColDP` works -- it is a classification-tree JSON, not a ColDP archive -- and it carries no synonym status either: 524,236 `accepted`, 2,933 `provisionally accepted`, zero `synonym`. The flat DwCA's own taxonomicStatus agrees -- 527,106 `accepted`, 21 `invalid`, and those 21 are the only rows where id != acceptedNameUsageID, pointing not to a synonym but to an obsolete 18th-century Linnaean group name (e.g. Clupeidae -&gt; "Abdominales Linnæus, 1758") -- noise, not synonymy. So the missing column is not an export-format gap to wait out: ZooBank's data model has no accepted/synonym concept to export, in any format ChecklistBank offers. Verdict unchanged, and nothing left to re-open on</t>
         </is>
       </c>
     </row>
     <row r="53" ht="60" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>checklistbank-310868</t>
+          <t>checklistbank-219318</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Tropicos (dataset 310868)</t>
+          <t>World Catalogue of the Tortricidae</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/dgrnm; version 2021, issued 2021-11-04</t>
+          <t>DOI 10.48580/d38s; version 4.0</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>https://api.checklistbank.org/dataset/310868/archive.zip</t>
+          <t>https://www.checklistbank.org/dataset/219318</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
@@ -2597,147 +2615,147 @@
           <t>CC BY</t>
         </is>
       </c>
-      <c r="F53" s="7" t="inlineStr">
+      <c r="F53" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>NOT taken. 1,368,229 name usages, 977,904 accepted species, and only 19.4% held over 20,580 measured -- the largest apparent gap in its batch, and declined anyway. It is 2021 data offered alongside a 2026 WFO list covering the same ground, so taking it would import older nomenclatural data over newer. Its 44.0% family coverage says most of what it offers is families WFO handles and we do not.</t>
+          <t>NOT taken. Found the same sweep, for our #13 gap family (Tortricidae, 12,239 missing). 10,718 accepted species, 10,678 of 10,685 normalised forms (99.9%) held, **7 new**. Declined; 2018 vintage adds nothing -- the gain is negligible regardless.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="60" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>eol-traitbank</t>
+          <t>checklistbank-310868</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>EOL TraitBank — all trait data</t>
+          <t>Tropicos (dataset 310868)</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.5281/zenodo.22129810</t>
+          <t>DOI 10.48580/dgrnm; version 2021, issued 2021-11-04</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>https://zenodo.org/records/22129810</t>
+          <t>https://api.checklistbank.org/dataset/310868/archive.zip</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>notspecified</t>
-        </is>
-      </c>
-      <c r="F54" s="7" t="inlineStr">
+          <t>CC BY</t>
+        </is>
+      </c>
+      <c r="F54" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>nothing yet. 11.4M trait rows, but values are ontology URIs rather than prose, and the licence is unspecified</t>
+          <t>NOT taken. 1,368,229 name usages, 977,904 accepted species, and only 19.4% held over 20,580 measured -- the largest apparent gap in its batch, and declined anyway. It is 2021 data offered alongside a 2026 WFO list covering the same ground, so taking it would import older nomenclatural data over newer. Its 44.0% family coverage says most of what it offers is families WFO handles and we do not.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="60" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>fishbase</t>
+          <t>eol-traitbank</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>FishBase (EOL harvest)</t>
+          <t>EOL TraitBank — all trait data</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.5281/zenodo.22739608</t>
+          <t>DOI 10.5281/zenodo.22129810</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>https://zenodo.org/records/22739608</t>
+          <t>https://zenodo.org/records/22129810</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>mixed; images are CC BY-NC 3.0</t>
-        </is>
-      </c>
-      <c r="F55" s="7" t="inlineStr">
+          <t>notspecified</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>NOT APPLIED, and nothing here is pending. English names measured: 28 marginal after GBIF vernacular, which is not a trade. Images are CC BY-NC 3.0 and refused. The separate ChecklistBank edition of FishBase (dataset 1010, CC BY) measured 100% already held over 600 of 600 sampled species. Nothing to do unless a policy question changes</t>
+          <t>nothing yet. 11.4M trait rows, but values are ontology URIs rather than prose, and the licence is unspecified</t>
         </is>
       </c>
     </row>
     <row r="56" ht="60" customHeight="1">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>gtdb</t>
+          <t>fishbase</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Genome Taxonomy Database r232</t>
+          <t>FishBase (EOL harvest)</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.15468/dpzg84 (GBIF dataset a97f36e5-ded1-49cc-bdec-ac6170fc7b9c); ColDP endpoint gtdb_r232_coldp.zip, issued 2026-08-25</t>
+          <t>DOI 10.5281/zenodo.22739608</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>https://hosted-datasets.gbif.org/gtdb/gtdb_r232_coldp.zip</t>
+          <t>https://zenodo.org/records/22739608</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
-        </is>
-      </c>
-      <c r="F56" s="7" t="inlineStr">
+          <t>mixed; images are CC BY-NC 3.0</t>
+        </is>
+      </c>
+      <c r="F56" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>DOWNLOADED AND READ, and it settles the question it was fetched for. 242,895 accepted name usages: 189,801 bacterial species in 3,967 families plus 10,122 archaeal, 125 phyla, two domains (Bacteria, Archaea) and no kingdom rank anywhere. That last fact is the one: COL's eight prokaryote clades -- Bacillati, Pseudomonadati, Thermotogati, Fusobacteriati, Methanobacteriati, Thermoproteati, Nanobdellati, Promethearchaeati -- return zero hits at any rank. They are not older spellings of GTDB names but a different convention (-ati where GTDB writes -ota) on the same organisms, ranked one level too high. COL's 'Bacillati' is GTDB's Bacillota, a phylum. So the tree's existing treatment of Archaea -- GTDB phyla such as Methanobacteriota and Thermoproteota as kingdom-rank nodes -- is the authority's own, and the bacteria question reduces to applying the same rule. Scope note: GTDB covers Bacteria and Archaea only and holds no viral taxa, so it says nothing about the virus half. See docs/bacteria-and-viruses.md.</t>
+          <t>NOT APPLIED, and nothing here is pending. English names measured: 28 marginal after GBIF vernacular, which is not a trade. Images are CC BY-NC 3.0 and refused. The separate ChecklistBank edition of FishBase (dataset 1010, CC BY) measured 100% already held over 600 of 600 sampled species. Nothing to do unless a policy question changes</t>
         </is>
       </c>
     </row>
     <row r="57" ht="60" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>ictv-msl</t>
+          <t>gtdb</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>ICTV Master Species List (MSL41)</t>
+          <t>Genome Taxonomy Database r232</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.5281/zenodo.19154110; published 2026-03-21; the 2025-2026 ICTV taxonomy, ratified February 2026</t>
+          <t>DOI 10.15468/dpzg84 (GBIF dataset a97f36e5-ded1-49cc-bdec-ac6170fc7b9c); ColDP endpoint gtdb_r232_coldp.zip, issued 2026-08-25</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>https://zenodo.org/records/19154110</t>
+          <t>https://hosted-datasets.gbif.org/gtdb/gtdb_r232_coldp.zip</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
@@ -2745,199 +2763,199 @@
           <t>CC BY 4.0</t>
         </is>
       </c>
-      <c r="F57" s="7" t="inlineStr">
+      <c r="F57" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>NOT DOWNLOADED, and deliberately so: viruses are on hold until further notice, so registering the source is the whole of the work for now. Recorded because it is the virus authority -- the one source that states the official ICTV taxonomy, which COL and Wikidata both decline to give at a usable rank. Two things to know before anyone does download it. It is an XLSX (ICTV_Master_Species_List_2025_MSL41.v1.xlsx, 1.80 MB), a fifth format this repo has no reader for, alongside NEWICK and DOT -- see docs/archive-formats.md. And sources/archives/ictv-msl/ exists but is EMPTY, left by an abandoned download, which is why this entry appears now rather than when the archive landed. Also CC BY 4.0, so citable with attribution once taken.</t>
+          <t>DOWNLOADED AND READ, and it settles the question it was fetched for. 242,895 accepted name usages: 189,801 bacterial species in 3,967 families plus 10,122 archaeal, 125 phyla, two domains (Bacteria, Archaea) and no kingdom rank anywhere. That last fact is the one: COL's eight prokaryote clades -- Bacillati, Pseudomonadati, Thermotogati, Fusobacteriati, Methanobacteriati, Thermoproteati, Nanobdellati, Promethearchaeati -- return zero hits at any rank. They are not older spellings of GTDB names but a different convention (-ati where GTDB writes -ota) on the same organisms, ranked one level too high. COL's 'Bacillati' is GTDB's Bacillota, a phylum. So the tree's existing treatment of Archaea -- GTDB phyla such as Methanobacteriota and Thermoproteota as kingdom-rank nodes -- is the authority's own, and the bacteria question reduces to applying the same rule. Scope note: GTDB covers Bacteria and Archaea only and holds no viral taxa, so it says nothing about the virus half. See docs/bacteria-and-viruses.md.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="60" customHeight="1">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>ncbi-taxonomy</t>
+          <t>ictv-msl</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>NCBI Taxonomy</t>
+          <t>ICTV Master Species List (MSL41)</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.15468/rhydar (GBIF dataset fab88965-e69d-4491-a04d-e3198b626e52, published 2026-04-17)</t>
+          <t>DOI 10.5281/zenodo.19154110; published 2026-03-21; the 2025-2026 ICTV taxonomy, ratified February 2026</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>https://www.gbif.org/dataset/fab88965-e69d-4491-a04d-e3198b626e52</t>
+          <t>https://zenodo.org/records/19154110</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>CC0</t>
-        </is>
-      </c>
-      <c r="F58" s="7" t="inlineStr">
+          <t>CC BY 4.0</t>
+        </is>
+      </c>
+      <c r="F58" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>overlap-measured 2026-10-08: 197,971 accepted species, 44,946 held (27.1%), 120,665 species not held (of which 1,853 are prokaryote/virus names on hold by decision). 3,120 of its 10,907 families are not in the tree. The only candidate that carries Bacteria and Viruses as real divisions with real authorities, which is exactly what COL will not give us: COL holds the prokaryotes and viruses in 17 clades at kingdom rank, so neither '--kingdom Bacteria' nor '--kingdom Viruses' reaches them (see docs/dataset-inbox.md). Against that, GBIF Backbone is already applied and is itself built from NCBI among others, so for the kingdoms we do hold this is largely a second copy of names we already have. Its value is narrower and real: prokaryote and viral coverage, and the type material and literature citations the NCBI record carries and no checklist we hold does. CC0, so licensing is not an obstacle. Not downloaded.</t>
+          <t>NOT DOWNLOADED, and deliberately so: viruses are on hold until further notice, so registering the source is the whole of the work for now. Recorded because it is the virus authority -- the one source that states the official ICTV taxonomy, which COL and Wikidata both decline to give at a usable rank. Two things to know before anyone does download it. It is an XLSX (ICTV_Master_Species_List_2025_MSL41.v1.xlsx, 1.80 MB), a fifth format this repo has no reader for, alongside NEWICK and DOT -- see docs/archive-formats.md. And sources/archives/ictv-msl/ exists but is EMPTY, left by an abandoned download, which is why this entry appears now rather than when the archive landed. Also CC BY 4.0, so citable with attribution once taken.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="60" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>species-fungorum</t>
+          <t>ncbi-taxonomy</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Species Fungorum Plus</t>
+          <t>NCBI Taxonomy</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.15468/ts7wsb</t>
+          <t>DOI 10.15468/rhydar (GBIF dataset fab88965-e69d-4491-a04d-e3198b626e52, published 2026-04-17)</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>https://www.gbif.org/dataset/bf3db7c9-5e5d-4fd0-bd5b-94539eaf9598</t>
+          <t>https://www.gbif.org/dataset/fab88965-e69d-4491-a04d-e3198b626e52</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
-        </is>
-      </c>
-      <c r="F59" s="7" t="inlineStr">
+          <t>CC0</t>
+        </is>
+      </c>
+      <c r="F59" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>nothing yet. 90% name match measured; 1,791 synonyms pending, and a checklist carries no descriptions</t>
+          <t>overlap-measured 2026-10-08: 197,971 accepted species, 44,946 held (27.1%), 120,665 species not held (of which 1,853 are prokaryote/virus names on hold by decision). 3,120 of its 10,907 families are not in the tree. The only candidate that carries Bacteria and Viruses as real divisions with real authorities, which is exactly what COL will not give us: COL holds the prokaryotes and viruses in 17 clades at kingdom rank, so neither '--kingdom Bacteria' nor '--kingdom Viruses' reaches them (see docs/dataset-inbox.md). Against that, GBIF Backbone is already applied and is itself built from NCBI among others, so for the kingdoms we do hold this is largely a second copy of names we already have. Its value is narrower and real: prokaryote and viral coverage, and the type material and literature citations the NCBI record carries and no checklist we hold does. CC0, so licensing is not an obstacle. Not downloaded.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="60" customHeight="1">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>taiwan-endemic</t>
+          <t>species-fungorum</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Endemic species in Taiwan</t>
+          <t>Species Fungorum Plus</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>GBIF DwCA, 3 members (taxon.txt)</t>
+          <t>DOI 10.15468/ts7wsb</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>(no DOI in the archive's eml.xml)</t>
+          <t>https://www.gbif.org/dataset/bf3db7c9-5e5d-4fd0-bd5b-94539eaf9598</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>CC0 1.0 (waived, per the eml.xml)</t>
-        </is>
-      </c>
-      <c r="F60" s="7" t="inlineStr">
+          <t>CC BY 4.0</t>
+        </is>
+      </c>
+      <c r="F60" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>NOT YET APPLIED, and assessed as narrow: 0.5 MB, one DwCA, endemic species of one island nation. Not a gap-filler -- it overlaps Taiwan material we already hold from COL and POWO. Worth taking only for the occurrence data if the distribution table carries it, which is the one thing here that is not a name we already have.</t>
+          <t>nothing yet. 90% name match measured; 1,791 synonyms pending, and a checklist carries no descriptions</t>
         </is>
       </c>
     </row>
     <row r="61" ht="60" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>usda-plants</t>
+          <t>taiwan-endemic</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>USDA PLANTS structured data</t>
+          <t>Endemic species in Taiwan</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>EOL harvest</t>
+          <t>GBIF DwCA, 3 members (taxon.txt)</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>https://zenodo.org/records/20646743</t>
+          <t>(no DOI in the archive's eml.xml)</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>notspecified</t>
-        </is>
-      </c>
-      <c r="F61" s="7" t="inlineStr">
+          <t>CC0 1.0 (waived, per the eml.xml)</t>
+        </is>
+      </c>
+      <c r="F61" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>nothing yet. 2,657 NativeRange records measured; values are Wikidata QIDs and GeoNames IDs needing resolution</t>
+          <t>NOT YET APPLIED, and assessed as narrow: 0.5 MB, one DwCA, endemic species of one island nation. Not a gap-filler -- it overlaps Taiwan material we already hold from COL and POWO. Worth taking only for the occurrence data if the distribution table carries it, which is the one thing here that is not a name we already have.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="60" customHeight="1">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>wikidata-species</t>
+          <t>usda-plants</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Wikidata Species (ChecklistBank dataset 314569)</t>
+          <t>USDA PLANTS structured data</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>DOI 10.48580/dgx38; version 2026-08-02; contact Markus Doering (GBIF); generated by CatalogueOfLife/coldp-generator</t>
+          <t>EOL harvest</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>https://www.checklistbank.org/dataset/314569</t>
+          <t>https://zenodo.org/records/20646743</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>CC0</t>
-        </is>
-      </c>
-      <c r="F62" s="7" t="inlineStr">
+          <t>notspecified</t>
+        </is>
+      </c>
+      <c r="F62" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>NOT IMPORTED, and not yet a decision either. Measured with scripts/overlapReport.py, which uses the importers' own held/new test rather than a raw string comparison: 3,207,163 accepted species, of which 1,395,018 (43.5%) we already hold and 1,811,989 (56.5%) are new. Of the new ones 91% resolve both a family and an order and would land in a real family rather than an Incertae sedis placeholder. Zero duplicates within the archive, 156 non-binomials. Taken, this would roughly double animalia and bring prokaryotes and viruses with it. CC0, so licensing is not an obstacle. It does NOT resolve the bacteria-and-viruses rank question: Wikidata carries the same 17 kingdom-rank clades COL does (Bacillati, Pseudomonadati, Orthornavirae, Heunggongvirae, ...) because it is built from the same upstream, and 1,612,751 of the new species have no parent at all. See docs/bacteria-and-viruses.md for the options. First archive in the ColDP format we hold, and first to exercise scripts/coldp.py. RE-CHECKED 2026-10-10: species-import question still correctly undecided -- it is downstream of the bacteria-and-viruses hold, which is unchanged (GTDB has since settled the bacterial rank; viruses are still blocked on ICTV). The 2026-10-04 measurement was already taken after Animalia Stage 2, so the ~135k species added since (ITIS, BOLD, GLI, Craneflies, Reptiles) shave a little off 1,811,989 but do not change the shape of the decision -- not worth re-measuring on its own. SIDECAR FINDING, measured 2026-10-10 against the held tree (scripts/tree.py, one walk, 2,531,312 held names): the same archive's sidecar tables carry real content the species-count note above never looked at, and most of each one lands on species we already hold -- this is an enrichment question, not an import one, so none of it waits on the bacteria-and-viruses hold. Media.tsv: 340,025 distinct taxa, 192,847 held, of which 110,224 already have an image in wiki-images.json and 82,623 do not -- but 663,287 of 664,930 rows (99.75%) carry no licence string at all, so that gap needs a per-image Commons licence lookup before anything is written, not a straight copy. VernacularName.tsv: 816,277 rows in 108 languages; filtered to en/blank the way scripts/enrichCommonNamesFromGbif.py filters GBIF's table, 95,067 distinct taxa, 70,935 held, 36,620 already have a commonName, **34,315 do not** -- a clean gap, larger than the 23,287 the already-applied GBIF Backbone pass filled, and the same safety pattern (empty-field-only, English-only, length/diagnosis filters) should carry over directly. Distribution.tsv: 293,850 rows, 103,213 distinct taxa, 66,815 held, 35,043 already have continents, 31,772 do not; 83.9% of rows are free-text place names needing resolution (the USDA PLANTS problem again) and 16.1% are ISO codes mappable through the existing CC2CONT table today -- roughly 5,100 of the 31,772 need no new plumbing. Not yet done: writing the importer. Vernacular is the obvious first pick -- biggest clean gap, smallest new code.</t>
+          <t>nothing yet. 2,657 NativeRange records measured; values are Wikidata QIDs and GeoNames IDs needing resolution</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2985,7 @@
           <t>CC BY 4.0</t>
         </is>
       </c>
-      <c r="F63" s="7" t="inlineStr">
+      <c r="F63" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
@@ -3004,7 +3022,7 @@
           <t>notspecified</t>
         </is>
       </c>
-      <c r="F64" s="7" t="inlineStr">
+      <c r="F64" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
@@ -3041,7 +3059,7 @@
           <t>open access registry; per-publication rights vary</t>
         </is>
       </c>
-      <c r="F65" s="7" t="inlineStr">
+      <c r="F65" s="8" t="inlineStr">
         <is>
           <t>assessed</t>
         </is>
@@ -3078,7 +3096,7 @@
           <t>CC BY-NC-SA 4.0</t>
         </is>
       </c>
-      <c r="F66" s="8" t="inlineStr">
+      <c r="F66" s="9" t="inlineStr">
         <is>
           <t>refused</t>
         </is>
@@ -3115,7 +3133,7 @@
           <t>CC BY-NC-SA 3.0</t>
         </is>
       </c>
-      <c r="F67" s="8" t="inlineStr">
+      <c r="F67" s="9" t="inlineStr">
         <is>
           <t>refused</t>
         </is>
@@ -3152,7 +3170,7 @@
           <t>CC BY-NC-SA 3.0</t>
         </is>
       </c>
-      <c r="F68" s="8" t="inlineStr">
+      <c r="F68" s="9" t="inlineStr">
         <is>
           <t>refused</t>
         </is>
@@ -3189,7 +3207,7 @@
           <t>mostly non-commercial per image</t>
         </is>
       </c>
-      <c r="F69" s="8" t="inlineStr">
+      <c r="F69" s="9" t="inlineStr">
         <is>
           <t>refused</t>
         </is>
@@ -3226,7 +3244,7 @@
           <t>ALL RIGHTS RESERVED</t>
         </is>
       </c>
-      <c r="F70" s="8" t="inlineStr">
+      <c r="F70" s="9" t="inlineStr">
         <is>
           <t>refused</t>
         </is>
@@ -3380,12 +3398,12 @@
           <t>2026-09</t>
         </is>
       </c>
-      <c r="L2" s="8" t="inlineStr">
+      <c r="L2" s="9" t="inlineStr">
         <is>
           <t>decline (probable)</t>
         </is>
       </c>
-      <c r="M2" s="8" t="inlineStr">
+      <c r="M2" s="9" t="inlineStr">
         <is>
           <t>decline (probable)</t>
         </is>
@@ -3680,12 +3698,12 @@
       <c r="I8" s="4" t="inlineStr"/>
       <c r="J8" s="4" t="inlineStr"/>
       <c r="K8" s="4" t="inlineStr"/>
-      <c r="L8" s="8" t="inlineStr">
+      <c r="L8" s="9" t="inlineStr">
         <is>
           <t>superseded — do not take</t>
         </is>
       </c>
-      <c r="M8" s="8" t="inlineStr">
+      <c r="M8" s="9" t="inlineStr">
         <is>
           <t>superseded — do not take</t>
         </is>
@@ -3952,12 +3970,12 @@
           <t>2005-11</t>
         </is>
       </c>
-      <c r="L15" s="8" t="inlineStr">
+      <c r="L15" s="9" t="inlineStr">
         <is>
           <t>do not take</t>
         </is>
       </c>
-      <c r="M15" s="8" t="inlineStr">
+      <c r="M15" s="9" t="inlineStr">
         <is>
           <t>do not take</t>
         </is>
@@ -4020,12 +4038,12 @@
           <t>2026-09</t>
         </is>
       </c>
-      <c r="L16" s="7" t="inlineStr">
+      <c r="L16" s="8" t="inlineStr">
         <is>
           <t>blocked on licence</t>
         </is>
       </c>
-      <c r="M16" s="7" t="inlineStr">
+      <c r="M16" s="8" t="inlineStr">
         <is>
           <t>blocked on licence</t>
         </is>
@@ -4204,12 +4222,12 @@
           <t>Oct 2017</t>
         </is>
       </c>
-      <c r="L19" s="8" t="inlineStr">
+      <c r="L19" s="9" t="inlineStr">
         <is>
           <t>do not take</t>
         </is>
       </c>
-      <c r="M19" s="8" t="inlineStr">
+      <c r="M19" s="9" t="inlineStr">
         <is>
           <t>do not take</t>
         </is>
@@ -4264,12 +4282,12 @@
           <t>Oct 2017</t>
         </is>
       </c>
-      <c r="L20" s="8" t="inlineStr">
+      <c r="L20" s="9" t="inlineStr">
         <is>
           <t>do not take</t>
         </is>
       </c>
-      <c r="M20" s="8" t="inlineStr">
+      <c r="M20" s="9" t="inlineStr">
         <is>
           <t>do not take</t>
         </is>
@@ -4324,12 +4342,12 @@
           <t>Oct 2026</t>
         </is>
       </c>
-      <c r="L21" s="8" t="inlineStr">
+      <c r="L21" s="9" t="inlineStr">
         <is>
           <t>decline</t>
         </is>
       </c>
-      <c r="M21" s="8" t="inlineStr">
+      <c r="M21" s="9" t="inlineStr">
         <is>
           <t>decline</t>
         </is>
@@ -4384,12 +4402,12 @@
           <t>Dec 2004</t>
         </is>
       </c>
-      <c r="L22" s="8" t="inlineStr">
+      <c r="L22" s="9" t="inlineStr">
         <is>
           <t>decline</t>
         </is>
       </c>
-      <c r="M22" s="8" t="inlineStr">
+      <c r="M22" s="9" t="inlineStr">
         <is>
           <t>decline</t>
         </is>
@@ -4444,12 +4462,12 @@
           <t>Jun 2005</t>
         </is>
       </c>
-      <c r="L23" s="8" t="inlineStr">
+      <c r="L23" s="9" t="inlineStr">
         <is>
           <t>decline</t>
         </is>
       </c>
-      <c r="M23" s="8" t="inlineStr">
+      <c r="M23" s="9" t="inlineStr">
         <is>
           <t>decline</t>
         </is>
@@ -4512,12 +4530,12 @@
           <t>2021</t>
         </is>
       </c>
-      <c r="L24" s="8" t="inlineStr">
+      <c r="L24" s="9" t="inlineStr">
         <is>
           <t>decline</t>
         </is>
       </c>
-      <c r="M24" s="8" t="inlineStr">
+      <c r="M24" s="9" t="inlineStr">
         <is>
           <t>decline</t>
         </is>
@@ -4780,12 +4798,12 @@
           <t>2021-06</t>
         </is>
       </c>
-      <c r="L28" s="8" t="inlineStr">
+      <c r="L28" s="9" t="inlineStr">
         <is>
           <t>decline</t>
         </is>
       </c>
-      <c r="M28" s="8" t="inlineStr">
+      <c r="M28" s="9" t="inlineStr">
         <is>
           <t>decline</t>
         </is>
@@ -4848,12 +4866,12 @@
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="L29" s="8" t="inlineStr">
+      <c r="L29" s="9" t="inlineStr">
         <is>
           <t>decline</t>
         </is>
       </c>
-      <c r="M29" s="8" t="inlineStr">
+      <c r="M29" s="9" t="inlineStr">
         <is>
           <t>decline</t>
         </is>
@@ -5056,12 +5074,12 @@
           <t>2017-08-25</t>
         </is>
       </c>
-      <c r="L32" s="8" t="inlineStr">
+      <c r="L32" s="9" t="inlineStr">
         <is>
           <t>decline</t>
         </is>
       </c>
-      <c r="M32" s="8" t="inlineStr">
+      <c r="M32" s="9" t="inlineStr">
         <is>
           <t>decline</t>
         </is>
@@ -5124,12 +5142,12 @@
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="L33" s="8" t="inlineStr">
+      <c r="L33" s="9" t="inlineStr">
         <is>
           <t>decline — see below</t>
         </is>
       </c>
-      <c r="M33" s="8" t="inlineStr">
+      <c r="M33" s="9" t="inlineStr">
         <is>
           <t>decline — see below</t>
         </is>

</xml_diff>